<commit_message>
Revert to pre-WalkIn state
</commit_message>
<xml_diff>
--- a/generated_invoices/36003-26.xlsx
+++ b/generated_invoices/36003-26.xlsx
@@ -1589,7 +1589,7 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" s="77" t="n"/>
       <c r="C5" s="77" t="n"/>
@@ -1604,7 +1604,7 @@
       <c r="H5" s="53" t="n"/>
       <c r="I5" s="91" t="inlineStr">
         <is>
-          <t>04-May-2026</t>
+          <t>06-Feb-2026</t>
         </is>
       </c>
       <c r="J5" s="92" t="n"/>
@@ -1646,7 +1646,7 @@
       <c r="H6" s="98" t="n"/>
       <c r="I6" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve"> - </t>
+          <t>12-Dec-2026</t>
         </is>
       </c>
       <c r="J6" s="92" t="n"/>
@@ -1792,7 +1792,7 @@
       <c r="B10" s="103" t="n"/>
       <c r="C10" s="103" t="inlineStr">
         <is>
-          <t>DEWA</t>
+          <t>TMZ</t>
         </is>
       </c>
       <c r="D10" s="84" t="n"/>
@@ -1883,7 +1883,7 @@
       <c r="B13" s="84" t="n"/>
       <c r="C13" s="67" t="inlineStr">
         <is>
-          <t>GSL/18730/26/AJM</t>
+          <t>LP/16732/26/DXB</t>
         </is>
       </c>
       <c r="D13" s="68" t="n"/>
@@ -1916,7 +1916,7 @@
       <c r="B14" s="84" t="n"/>
       <c r="C14" s="79" t="inlineStr">
         <is>
-          <t>Al Quoz</t>
+          <t>Dubai</t>
         </is>
       </c>
       <c r="D14" s="81" t="n"/>
@@ -1949,7 +1949,7 @@
       <c r="B15" s="39" t="n"/>
       <c r="C15" s="79" t="inlineStr">
         <is>
-          <t>Test 2</t>
+          <t xml:space="preserve">material tests </t>
         </is>
       </c>
       <c r="D15" s="43" t="n"/>
@@ -2066,40 +2066,36 @@
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
         <is>
-          <t>GR - 040326 - 005</t>
+          <t>GR - 060226 - 001</t>
         </is>
       </c>
       <c r="B18" s="127" t="inlineStr">
         <is>
-          <t>04-Mar-2026</t>
+          <t>06-Feb-2026</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>34567ASDFGHJK</t>
+          <t>12393JSDN</t>
         </is>
       </c>
       <c r="D18" s="109" t="inlineStr">
         <is>
-          <t>Loss of Stability of Compacted Bituminous Mixtures Using Marshall Apparatus.</t>
-        </is>
-      </c>
-      <c r="E18" s="110" t="inlineStr">
-        <is>
-          <t>DM 10</t>
-        </is>
-      </c>
+          <t>Mobilization &amp; Demobilization</t>
+        </is>
+      </c>
+      <c r="E18" s="110" t="inlineStr"/>
       <c r="F18" s="110" t="n"/>
       <c r="G18" s="110" t="n"/>
       <c r="H18" s="111" t="n"/>
       <c r="I18" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" s="112" t="n">
-        <v>125</v>
+        <v>1000</v>
       </c>
       <c r="K18" s="112" t="n">
-        <v>125</v>
+        <v>2000</v>
       </c>
       <c r="L18" s="7" t="n"/>
       <c r="M18" s="7" t="n"/>
@@ -2115,39 +2111,17 @@
       <c r="W18" s="7" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="66" t="inlineStr">
-        <is>
-          <t>GR - 040326 - 006</t>
-        </is>
-      </c>
-      <c r="B19" s="128" t="inlineStr">
-        <is>
-          <t>04-Mar-2026</t>
-        </is>
-      </c>
+      <c r="A19" s="66" t="n"/>
+      <c r="B19" s="128" t="n"/>
       <c r="C19" s="66" t="n"/>
-      <c r="D19" s="113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Marshall Stability &amp; Flow of Bituminous Mixture </t>
-        </is>
-      </c>
-      <c r="E19" s="114" t="inlineStr">
-        <is>
-          <t>ASTM D 6927</t>
-        </is>
-      </c>
+      <c r="D19" s="113" t="n"/>
+      <c r="E19" s="114" t="n"/>
       <c r="F19" s="114" t="n"/>
       <c r="G19" s="114" t="n"/>
       <c r="H19" s="115" t="n"/>
-      <c r="I19" s="66" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="116" t="n">
-        <v>100</v>
-      </c>
-      <c r="K19" s="116" t="n">
-        <v>100</v>
-      </c>
+      <c r="I19" s="66" t="n"/>
+      <c r="J19" s="116" t="n"/>
+      <c r="K19" s="116" t="n"/>
       <c r="L19" s="7" t="n"/>
       <c r="M19" s="7" t="n"/>
       <c r="N19" s="7" t="n"/>
@@ -2566,8 +2540,9 @@
       <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
       <c r="J35" s="10" t="n"/>
-      <c r="K35" s="47" t="n">
-        <v>225</v>
+      <c r="K35" s="47">
+        <f>SUM(K18:K18)</f>
+        <v/>
       </c>
       <c r="L35" s="7" t="n"/>
       <c r="M35" s="7" t="n"/>
@@ -2601,8 +2576,9 @@
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
       <c r="J36" s="10" t="n"/>
-      <c r="K36" s="47" t="n">
-        <v>11.25</v>
+      <c r="K36" s="47">
+        <f>K35*0.05</f>
+        <v/>
       </c>
       <c r="L36" s="7" t="n"/>
       <c r="M36" s="7" t="n"/>
@@ -2636,8 +2612,9 @@
       <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
       <c r="J37" s="10" t="n"/>
-      <c r="K37" s="51" t="n">
-        <v>236.25</v>
+      <c r="K37" s="51">
+        <f>K35+K36</f>
+        <v/>
       </c>
       <c r="L37" s="7" t="n"/>
       <c r="M37" s="7" t="n"/>
@@ -2660,7 +2637,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Two Hundred Thirty Six Dirhams and Twenty Five Fils Only</t>
+          <t>Two Thousand and One Hundred Dirhams Only</t>
         </is>
       </c>
       <c r="C38" s="85" t="n"/>

</xml_diff>